<commit_message>
demo product set, polished product pages with links
</commit_message>
<xml_diff>
--- a/scripture-creations/catalog.xlsx
+++ b/scripture-creations/catalog.xlsx
@@ -2,41 +2,30 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Websites\Reed\scripture-creations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScriptureCreations\Marketing\WebSite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A78718-99B5-46B4-A1DA-48784639EB14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F5E7B5-6DC4-483F-9AD4-753E16263C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{82252E67-CF23-4A4C-8DD5-12847BD7CFFE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="79">
   <si>
     <t>id</t>
   </si>
@@ -53,69 +42,12 @@
     <t>image</t>
   </si>
   <si>
-    <t>BoxArticles.jpg</t>
-  </si>
-  <si>
-    <t>games</t>
-  </si>
-  <si>
-    <t>Articles of Faith Memorization Game</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>Here is an example description.</t>
-  </si>
-  <si>
-    <t>sku_001</t>
-  </si>
-  <si>
-    <t>sku_002</t>
-  </si>
-  <si>
     <t>Book of Mormon Chronology Bookmark</t>
   </si>
   <si>
-    <t>bookmarks</t>
-  </si>
-  <si>
-    <t>BofMBookmark.jpg</t>
-  </si>
-  <si>
-    <t>Here is an example description 2.</t>
-  </si>
-  <si>
-    <t>sku_003</t>
-  </si>
-  <si>
-    <t>"Hold up your light" Graphic</t>
-  </si>
-  <si>
-    <t>posters</t>
-  </si>
-  <si>
-    <t>HoldupLight.jpg</t>
-  </si>
-  <si>
-    <t>Here is an example description 3.</t>
-  </si>
-  <si>
-    <t>sku_004</t>
-  </si>
-  <si>
-    <t>Missionary Journey Legend</t>
-  </si>
-  <si>
-    <t>other</t>
-  </si>
-  <si>
-    <t>Missionary Legend.jpg</t>
-  </si>
-  <si>
-    <t>Here is an example description 4.</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -126,6 +58,210 @@
   </si>
   <si>
     <t>is_featured</t>
+  </si>
+  <si>
+    <t>Signs of the Times Pamphlet</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>This pamphlet lists 300+ signs of the times from the LDS scriptures in chronological order including most of the associated scriptures. It uses the Book of Revelation as a base and merges all the other scriptures in trying to keep the events in the order they are mentioned by each prophet.</t>
+  </si>
+  <si>
+    <t>Signs Pamphlet.jpg</t>
+  </si>
+  <si>
+    <t>Signs of the Times Chart</t>
+  </si>
+  <si>
+    <t>SignsOfTimes.jpg</t>
+  </si>
+  <si>
+    <t>This chart shows 129 prophecies in relationship to the church, the house of Israel, and the world in general.  A concise overview of the times we are living in and the signs of the second coming of Jesus Christ.  Laminated.</t>
+  </si>
+  <si>
+    <t>Missionary Pack (9 bookmarks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Includes: Plan of Salvation, Evidences for Joseph Smith, Evidences for the B. of M., Points of Christ’s True Church, Prophecies Fulfilled by Jesus Christ, Daniel’s Vision of the Restoration, Introduction to The Church of Jesus Christ of Latter-day Saints, Eternal Rewards, LDS Doctrine of Deity, and Book of Mormon study map. </t>
+  </si>
+  <si>
+    <t>Doctrine of Deity Pamphlet.jpg</t>
+  </si>
+  <si>
+    <t>Book of Mormon Study Map Bookmark</t>
+  </si>
+  <si>
+    <t>Book of Mormon</t>
+  </si>
+  <si>
+    <t>BofMTimeLineFront.jpg</t>
+  </si>
+  <si>
+    <t>A time line of Book of Mormon events and people.  Has the authors of the Books in the Book of Mormon and when they wrote.  Has a quick reference for the major stories, events, and quoted scriptures in the Book of Mormon.  Laminated.</t>
+  </si>
+  <si>
+    <t>Genealogy of the 12 Tribes Bookmark</t>
+  </si>
+  <si>
+    <t>Old Testament</t>
+  </si>
+  <si>
+    <t>Genealogy of 12 Tribes Sm.jpg</t>
+  </si>
+  <si>
+    <t>Shows family relationships for Abraham, Isaac, Jacob, &amp; his sons.  Shows from whom the Moabites, Edomites, &amp; Children of Ammon descended.  The back defines the Abrahamic covenant.  Laminated.</t>
+  </si>
+  <si>
+    <t>Old Testament Chrolonology Bookmark</t>
+  </si>
+  <si>
+    <t>OTBookmarkFront.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark shows a time line of Old Testament events and people.  It shows the patriarchs' births and how long they lived.  Identifies roles of the leaders in Israel and Judah.  Laminated.</t>
+  </si>
+  <si>
+    <t>New Testament Study Map Bookmark</t>
+  </si>
+  <si>
+    <t>New Testament</t>
+  </si>
+  <si>
+    <t>NTMap.jpg</t>
+  </si>
+  <si>
+    <t>New Testament Study Map Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A 8.5 x 11" map of the New Testament area with pictures of many events of Christ's life at the locations where they happened.  The Map lists all of Jesus Christ's parables, miracles, and events.  Laminated. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A 4.75" x 7" map of the New Testament area with pictures of many events of Christ's life at the locations where they happened.  Laminated. </t>
+  </si>
+  <si>
+    <t>Parables of Jesus Christ Bookmark</t>
+  </si>
+  <si>
+    <t>ParablesSm.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark lists all the parables of Jesus Christ that are recorded in the New Testament with their references.   Laminated.</t>
+  </si>
+  <si>
+    <t>Miracles of Jesus Christ</t>
+  </si>
+  <si>
+    <t>MiraclesOfJesusChristBackground.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark lists all the miracles Jesus performed that are recorded in the New Testament with their references.    Laminated</t>
+  </si>
+  <si>
+    <t>Revelations Condensed Bookmark</t>
+  </si>
+  <si>
+    <t>Revelations Condensed.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark condenses the Book of Revelations to provide a list of 107 events leading up to Christ's second coming.  Laminated.</t>
+  </si>
+  <si>
+    <t>Book of Mormon and the American Indian Chart</t>
+  </si>
+  <si>
+    <t>BofM-Indians.jpg</t>
+  </si>
+  <si>
+    <t>This 8.5" x 11" Chart combines the prophecies about the American Indians into one concice chart.  Who are they?  Prophecies of the gentiles coming.  Why were they destroyed as a people?  What is their future?  Laminated.</t>
+  </si>
+  <si>
+    <t>Plan of Salvation Bookmark</t>
+  </si>
+  <si>
+    <t>PlanOFSalvation.jpg</t>
+  </si>
+  <si>
+    <t>A 4.75" x 7" bookmark showing a detailed plan of salvation chart with a time line of the major events of this earth.  The back contains the associated scripture references.  Laminated.</t>
+  </si>
+  <si>
+    <t>Plan of Salvation Chart</t>
+  </si>
+  <si>
+    <t>A 8.5" x 11" chart showing the plan of salvation with a time line of the major events of this earth.  The back contains the associated scripture references.  Laminated.</t>
+  </si>
+  <si>
+    <t>Doctrine of Deity Bookmark</t>
+  </si>
+  <si>
+    <t>This 4.75" x 7z' bookmark shows that the Church of Jesus Christ of Latter-day Saints’ Doctrine of Deity is biblical. It lists over 150 scriptures showing the Godhead is three distinct persons, men are God’s children and can become like him, etc.  Laminated.</t>
+  </si>
+  <si>
+    <t>Church History Study Map Bookmark</t>
+  </si>
+  <si>
+    <t>Doctrine and Covenants</t>
+  </si>
+  <si>
+    <t>ChMap.jpg</t>
+  </si>
+  <si>
+    <t>Church History Study Map Chart</t>
+  </si>
+  <si>
+    <t>A 8.5z' x 11" map of the United States with locations and events that transpired as church history unfolded.  It shows where each section of the D&amp;C was recieved. The back has the chronology of the early church history.  Laminated.</t>
+  </si>
+  <si>
+    <t>A 4.75" x 7" map of the United States with locations and events that transpired as church history unfolded.  It shows where each section of the D&amp;C was recieved. The back has the chronology of the early church history.  Laminated.</t>
+  </si>
+  <si>
+    <t>Eternal Rewards Bookmark</t>
+  </si>
+  <si>
+    <t>EternalRewards.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark summarizes D&amp;C 76 and contrasts the  telestial, terrestrial, and celestial kingdoms and shows the requirements and rewards for each kingdom.  Laminated.</t>
+  </si>
+  <si>
+    <t>Evidences for Joseph Smith Bookmark</t>
+  </si>
+  <si>
+    <t>EvidencesForJSMarketingSmall.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark lists many of the things that Joseph Smith did that are evidences that he truly was a prophet of God.   Laminated.</t>
+  </si>
+  <si>
+    <t>Book of Mormon Study Map Chart</t>
+  </si>
+  <si>
+    <t>4.75" x 7" bookmark with a map of the relative geography of the Book of Mormon.  All 8.5" x 11" chart with a map have a gazetteer on the back to help find locations. Laminated.</t>
+  </si>
+  <si>
+    <t>8.5" x 11" map of the relative geography of the Book of Mormon.  Map have a gazetteer on the back to help find locations. Laminated.</t>
+  </si>
+  <si>
+    <t>Book of Mormon Study Map Companion</t>
+  </si>
+  <si>
+    <t>Wallmap5x7.jpg</t>
+  </si>
+  <si>
+    <t>Book of Mormon Companion.jpg</t>
+  </si>
+  <si>
+    <t>Genealogy of the 12 Tribes Chart</t>
+  </si>
+  <si>
+    <t>Yard Signs of Jesus</t>
+  </si>
+  <si>
+    <t>Box Top.jpg</t>
+  </si>
+  <si>
+    <t>10 beautiful 12" x 18" yard signs with H-stakes showing images of Jesus. Great for showing your love for Jesus Christ ($15 per image)</t>
   </si>
 </sst>
 </file>
@@ -511,11 +647,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7BF97CC-7DEE-4464-A48F-5AD6090A9F53}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="13.109375" customWidth="1"/>
+    <col min="2" max="2" width="35.77734375" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="20.33203125" customWidth="1"/>
+    <col min="5" max="5" width="31.5546875" customWidth="1"/>
     <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="72.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -535,117 +676,637 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>67057900453</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>67057900451</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>67057900550</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1">
+        <v>19.95</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>67057900403</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>67057900401</v>
+      </c>
+      <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="1">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>67057900402</v>
+      </c>
+      <c r="B7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="1">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>67057900420</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" t="s">
+        <v>5</v>
+      </c>
+      <c r="H8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>67057900486</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="F9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>67057900487</v>
+      </c>
+      <c r="B10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="1">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>67057900425</v>
+      </c>
+      <c r="B11" t="s">
         <v>29</v>
       </c>
-      <c r="H1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C11" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" t="s">
+        <v>5</v>
+      </c>
+      <c r="G11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>67057900441</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" t="s">
+        <v>5</v>
+      </c>
+      <c r="H12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>67057900440</v>
+      </c>
+      <c r="B13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="1">
+        <v>6</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="H13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>67057900435</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" t="s">
+        <v>5</v>
+      </c>
+      <c r="G14" t="s">
+        <v>7</v>
+      </c>
+      <c r="H14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>67057900437</v>
+      </c>
+      <c r="B15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" t="s">
+        <v>7</v>
+      </c>
+      <c r="H15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>67057900484</v>
+      </c>
+      <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" t="s">
+        <v>7</v>
+      </c>
+      <c r="H16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>67057900416</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="1">
         <v>6</v>
       </c>
-      <c r="E2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="D17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G17" t="s">
+        <v>7</v>
+      </c>
+      <c r="H17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>67057900456</v>
+      </c>
+      <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D18" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="1">
-        <v>4</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="1">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="E18" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18" t="s">
+        <v>5</v>
+      </c>
+      <c r="G18" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>67057900458</v>
+      </c>
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="1">
+        <v>6</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" t="s">
+        <v>5</v>
+      </c>
+      <c r="G19" t="s">
+        <v>5</v>
+      </c>
+      <c r="H19" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>67057900414</v>
+      </c>
+      <c r="B20" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" t="s">
-        <v>25</v>
+      <c r="F20" t="s">
+        <v>5</v>
+      </c>
+      <c r="G20" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>67057900444</v>
+      </c>
+      <c r="B21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F21" t="s">
+        <v>5</v>
+      </c>
+      <c r="G21" t="s">
+        <v>7</v>
+      </c>
+      <c r="H21" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>67057900443</v>
+      </c>
+      <c r="B22" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" s="1">
+        <v>6</v>
+      </c>
+      <c r="D22" t="s">
+        <v>58</v>
+      </c>
+      <c r="E22" t="s">
+        <v>59</v>
+      </c>
+      <c r="F22" t="s">
+        <v>5</v>
+      </c>
+      <c r="G22" t="s">
+        <v>7</v>
+      </c>
+      <c r="H22" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>67057900482</v>
+      </c>
+      <c r="B23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D23" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" t="s">
+        <v>64</v>
+      </c>
+      <c r="F23" t="s">
+        <v>5</v>
+      </c>
+      <c r="G23" t="s">
+        <v>7</v>
+      </c>
+      <c r="H23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>67057900461</v>
+      </c>
+      <c r="B24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E24" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" t="s">
+        <v>5</v>
+      </c>
+      <c r="G24" t="s">
+        <v>7</v>
+      </c>
+      <c r="H24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>67057900461</v>
+      </c>
+      <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="1">
+        <v>150</v>
+      </c>
+      <c r="D25" t="s">
+        <v>33</v>
+      </c>
+      <c r="E25" t="s">
+        <v>77</v>
+      </c>
+      <c r="F25" t="s">
+        <v>5</v>
+      </c>
+      <c r="G25" t="s">
+        <v>5</v>
+      </c>
+      <c r="H25" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
email cleaned, purchase page cleaned
</commit_message>
<xml_diff>
--- a/scripture-creations/catalog.xlsx
+++ b/scripture-creations/catalog.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScriptureCreations\Marketing\WebSite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F5E7B5-6DC4-483F-9AD4-753E16263C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA78F98C-E9CC-4D17-BE28-02B8C2DDD663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{82252E67-CF23-4A4C-8DD5-12847BD7CFFE}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82252E67-CF23-4A4C-8DD5-12847BD7CFFE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="162">
   <si>
     <t>id</t>
   </si>
@@ -261,7 +262,256 @@
     <t>Box Top.jpg</t>
   </si>
   <si>
-    <t>10 beautiful 12" x 18" yard signs with H-stakes showing images of Jesus. Great for showing your love for Jesus Christ ($15 per image)</t>
+    <t>Games</t>
+  </si>
+  <si>
+    <t>Articles of Faith Memorization Game</t>
+  </si>
+  <si>
+    <t>ArticlesBox.jpg</t>
+  </si>
+  <si>
+    <t>A card game to help memorize the Articles of Faith.  Each Article of Faith card has a picture clue to help with memorization.  Includes a die and a brief history of the Articles of Faith.</t>
+  </si>
+  <si>
+    <t>Fishing for Nephites Game (go fish)</t>
+  </si>
+  <si>
+    <t>FishingBox.jpg</t>
+  </si>
+  <si>
+    <t>Play "Fish" using pictures of events that transpired in the Book of Mormon.  Teaches names of characters in the Book of Mormon and events.  Cards are UV coated for durability.</t>
+  </si>
+  <si>
+    <t>The Frugal Family Game</t>
+  </si>
+  <si>
+    <t>FrugalFamily.jpg</t>
+  </si>
+  <si>
+    <t>Players are each given a dollar and watch it dwindle as the lights are left on, food is wasted, water bills rise, possessions are not taken care of, etc.  Helps family members learn that money is either saved or wasted depending on the choices they make.  Comes with eight pawns.  Laminated.</t>
+  </si>
+  <si>
+    <t>Abrahamic Covenant Chart</t>
+  </si>
+  <si>
+    <t>AbrahamicCovenantMarketing.jpg</t>
+  </si>
+  <si>
+    <t>This chart explains the Abrahamic Covenant, who it is to and what it is.   Laminated.</t>
+  </si>
+  <si>
+    <t>The Lost 10 Tribes Chart</t>
+  </si>
+  <si>
+    <t>LostTribesMarketing.jpg</t>
+  </si>
+  <si>
+    <t>This chart lists what we know of the lost tribes, where they went, where they are, when and how will they return.   Laminated.</t>
+  </si>
+  <si>
+    <t>Miracles of the Old Testament Bookmark</t>
+  </si>
+  <si>
+    <t>Miracles of the OT.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark lists the miracles recorded in the Old Testament with their scripture references.  Laminated.</t>
+  </si>
+  <si>
+    <t>Events of the Old Testament Bookmark</t>
+  </si>
+  <si>
+    <t>events-of-the-old-testament-bookmark.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark is designed as a quick reference for major events that happened in the Old Testament and their scripture references.  Laminated.</t>
+  </si>
+  <si>
+    <t>Daniel's Vision of the Restoration Bookmark</t>
+  </si>
+  <si>
+    <t>Daniels Vision.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark shows how Daniel saw the year when Joseph Smith would complete the restoration and “the sanctuary” would be cleansed.    Laminated.</t>
+  </si>
+  <si>
+    <t>Prophecies Fulfilled by Jesus Christ Bkmrk</t>
+  </si>
+  <si>
+    <t>PropheciesOfChristMarketing.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark lists many of the prophecies about Jesus Christ recorded in the Old Testament with their scripture references.  Laminated.</t>
+  </si>
+  <si>
+    <t>Events of the New Testament Bookmark</t>
+  </si>
+  <si>
+    <t>NTEvents.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark lists many major events in the New Testament, their locations, and the scripture reference.    Laminated.</t>
+  </si>
+  <si>
+    <t>Points of Christ's True Church Bookmark</t>
+  </si>
+  <si>
+    <t>Points of Christs True Church.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark lists 48 doctrines that were taught by Jesus and his disciples that should exist in His church today.  All references are from the Bible.  Laminated.</t>
+  </si>
+  <si>
+    <t>10 beautiful 12" x 18" yard signs with H-stakes showing images of Jesus. Great for showing your love for Jesus Christ at Christmas, Easter, or anytime.  ($15 per sign)</t>
+  </si>
+  <si>
+    <t>Evidences for the Book of Mormon Bookmark</t>
+  </si>
+  <si>
+    <t>EvidencesForBofMMarketing.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark lists many of the evidences for the Book of Mormon.  Laminated.</t>
+  </si>
+  <si>
+    <t>Miracles of the Book of Mormon Bookmark</t>
+  </si>
+  <si>
+    <t>Book of Mormon Miracles.jpg</t>
+  </si>
+  <si>
+    <t>Lists many of the miracles spoken of in the Book of Mormon.  Laminated.</t>
+  </si>
+  <si>
+    <t>People of the Book of Mormon Chart</t>
+  </si>
+  <si>
+    <t>People of BofM.jpg</t>
+  </si>
+  <si>
+    <t>List all the people in the Book of Mormon (non-Jaradite) in the chronological order they are mentioned.  It indicates their main roles and affiliations.  A great Book of Mormon overview and study help. Laminated.</t>
+  </si>
+  <si>
+    <t>QuickReferenceMarketingSm.jpg</t>
+  </si>
+  <si>
+    <t>A bookmark that lists church doctrine and oft quoted scriptures and where to find them in the Doctrine and Covenants.  Laminated.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doctrine and Covenants Quick Reference Bookmark </t>
+  </si>
+  <si>
+    <t>Priesthood Offices, Quorums and Duties Bookmark</t>
+  </si>
+  <si>
+    <t>PriesthoodSm.jpg</t>
+  </si>
+  <si>
+    <t>This bookmark lists the offices, quorums, and duties of the Aaronic &amp; Melchizedek Priesthood and includes the scripture references associated with each office.  Laminated.</t>
+  </si>
+  <si>
+    <t>Evidences for Joseph Smith &amp; Book of Mormon</t>
+  </si>
+  <si>
+    <t>PlaceMatJSEvidencesMarketing.jpg</t>
+  </si>
+  <si>
+    <t>Shows many evidences why Joseph Smith was a prophet and why the Book of Mormon is a true book of scripture.  One side shows the evidences for Joseph Smith and the other shows evidences for the Book of Mormon. Great teaching chart for Sunday School, Seminary, and Family Home Evening. Can be used as a placemat to strengthen faith every morning.  Laminated.</t>
+  </si>
+  <si>
+    <t>Introduction to the Church of Jesus Christ of Latter-day Saints Bookmark</t>
+  </si>
+  <si>
+    <t>This bookmark is designed as a pass along card to share LDS beliefs with those who would like to know more about the Church of Jesus Christ of Latter-day Saints. Laminated.</t>
+  </si>
+  <si>
+    <t>Introduction to the Church of Jesus Christ of Latter-day Saints 10-pack</t>
+  </si>
+  <si>
+    <t>2500 Signs of the Times in Chronological Order ebook</t>
+  </si>
+  <si>
+    <t>Ri Conquers the Multiverse ebook</t>
+  </si>
+  <si>
+    <t>Criticism to Gratitude Tracker Chart</t>
+  </si>
+  <si>
+    <t>Book of Mormon Study Map Wall Chart</t>
+  </si>
+  <si>
+    <t>19" x 26" wall map of the relative geography of the Book of Mormon.  Map have a gazetteer and scriptures mentioning each location on the back to help find locations. Laminated.</t>
+  </si>
+  <si>
+    <t>These cards are designed to share LDS beliefs with those who would like to know more about the Church of Jesus Christ of Latter-day Saints. Pack of 10 cards to leave out on your desk or wherever those interested can find them or pass along to someone who might be interested.  Laminated.</t>
+  </si>
+  <si>
+    <t>Picture Puzzle</t>
+  </si>
+  <si>
+    <t>2500Signs.jpg</t>
+  </si>
+  <si>
+    <t>Introduction to Church.jpg</t>
+  </si>
+  <si>
+    <t>Images of Jesus Coloring Book</t>
+  </si>
+  <si>
+    <t>Getting Satan Out of Your Marriage Pamphlet</t>
+  </si>
+  <si>
+    <t>Deep State in the Book of Mormon</t>
+  </si>
+  <si>
+    <t>RiFinal.jpg</t>
+  </si>
+  <si>
+    <t>Deep State Image.jpg</t>
+  </si>
+  <si>
+    <t>MarriagePamphlet.jpeg</t>
+  </si>
+  <si>
+    <t>This book gives a comprehensive list of scriptures about future events. It takes Revelation, Mathew 24, Luke 20, and JS Mathew as a skeleton and adds in all the other references attempting to keep them in the order given in each chapter. Great for a deep dive into the Signs of Christ's coming.</t>
+  </si>
+  <si>
+    <t>The Deep State, Secret Combinations, is talked about more in the Book of Mormon than America being a choice land. Why did Moroni warn us of this threat? How can we identify them?</t>
+  </si>
+  <si>
+    <t>Coloring book with 20 pictures and titles of Jesus. 8.5" x 11"</t>
+  </si>
+  <si>
+    <t>10 pictures of Jesus with small snips from the pictures to match with the pictures, with three levels of dificulty.</t>
+  </si>
+  <si>
+    <t>Shouldn't marital problems be solved through the gospel of Jesus Christ? How much of the conflict comes from not being Christ-like? This is a two week program to catapult your relationship from frustrating to fantastic.</t>
+  </si>
+  <si>
+    <t>How happy can you be? Non-judgmental, non-critical, forgiving, and grateful make for a happy marriage and life. This is a chart for helping move your life to amazing. "whoso is happy, will be happy still…." --Mormon 9:14</t>
+  </si>
+  <si>
+    <t>A ward challenge. Can you do the temple work for enough people to fill a spirit world chapel? Add a dot for each ordinance done and see their chapel fill.</t>
+  </si>
+  <si>
+    <t>Follow a young intelligence as he learns and grows while moving through worlds of his progression. A little "coming of age", a little "a boy and his dog" and a little romance. "Ri Conquers the Multiverse" will change your view your life.</t>
+  </si>
+  <si>
+    <t>Fill a Spirit Ward</t>
+  </si>
+  <si>
+    <t>Coloring Book Front for Marketing.jpg</t>
+  </si>
+  <si>
+    <t>Fill a Chapel.jpg</t>
+  </si>
+  <si>
+    <t>Front Page - Criticism to Gratitude.jpg</t>
+  </si>
+  <si>
+    <t>Puzzle 1 Cover.jpg</t>
   </si>
 </sst>
 </file>
@@ -647,16 +897,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7BF97CC-7DEE-4464-A48F-5AD6090A9F53}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" customWidth="1"/>
-    <col min="2" max="2" width="35.77734375" customWidth="1"/>
+    <col min="2" max="2" width="57.21875" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" style="1"/>
     <col min="4" max="4" width="20.33203125" customWidth="1"/>
-    <col min="5" max="5" width="31.5546875" customWidth="1"/>
+    <col min="5" max="5" width="33.21875" customWidth="1"/>
     <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="72.21875" customWidth="1"/>
+    <col min="8" max="8" width="201.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -817,19 +1067,19 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>67057900402</v>
+        <v>67057900410</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>137</v>
       </c>
       <c r="C7" s="1">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
         <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F7" t="s">
         <v>5</v>
@@ -838,50 +1088,50 @@
         <v>7</v>
       </c>
       <c r="H7" t="s">
-        <v>70</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>67057900420</v>
+        <v>67057900402</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>72</v>
       </c>
       <c r="C8" s="1">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="F8" t="s">
         <v>5</v>
       </c>
       <c r="G8" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H8" t="s">
-        <v>24</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>67057900486</v>
+        <v>67057900420</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="C9" s="1">
         <v>3.5</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F9" t="s">
         <v>5</v>
@@ -890,18 +1140,18 @@
         <v>5</v>
       </c>
       <c r="H9" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>67057900487</v>
+        <v>67057900486</v>
       </c>
       <c r="B10" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="C10" s="1">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="D10" t="s">
         <v>26</v>
@@ -921,19 +1171,19 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>67057900425</v>
+        <v>67057900487</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="C11" s="1">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="D11" t="s">
         <v>26</v>
       </c>
       <c r="E11" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F11" t="s">
         <v>5</v>
@@ -942,24 +1192,24 @@
         <v>5</v>
       </c>
       <c r="H11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>67057900441</v>
+        <v>67057900425</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C12" s="1">
         <v>3.5</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F12" t="s">
         <v>5</v>
@@ -968,18 +1218,18 @@
         <v>5</v>
       </c>
       <c r="H12" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>67057900440</v>
+        <v>67057900441</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C13" s="1">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="D13" t="s">
         <v>33</v>
@@ -991,27 +1241,27 @@
         <v>5</v>
       </c>
       <c r="G13" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>67057900435</v>
+        <v>67057900440</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C14" s="1">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="D14" t="s">
         <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
         <v>5</v>
@@ -1020,15 +1270,15 @@
         <v>7</v>
       </c>
       <c r="H14" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>67057900437</v>
+        <v>67057900435</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C15" s="1">
         <v>3.5</v>
@@ -1037,7 +1287,7 @@
         <v>33</v>
       </c>
       <c r="E15" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F15" t="s">
         <v>5</v>
@@ -1046,15 +1296,15 @@
         <v>7</v>
       </c>
       <c r="H15" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>67057900484</v>
+        <v>67057900437</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C16" s="1">
         <v>3.5</v>
@@ -1063,7 +1313,7 @@
         <v>33</v>
       </c>
       <c r="E16" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F16" t="s">
         <v>5</v>
@@ -1072,24 +1322,24 @@
         <v>7</v>
       </c>
       <c r="H16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>67057900416</v>
+        <v>67057900484</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C17" s="1">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="D17" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E17" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F17" t="s">
         <v>5</v>
@@ -1098,44 +1348,44 @@
         <v>7</v>
       </c>
       <c r="H17" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>67057900456</v>
+        <v>67057900416</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C18" s="1">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="D18" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F18" t="s">
         <v>5</v>
       </c>
       <c r="G18" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H18" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>67057900458</v>
+        <v>67057900456</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C19" s="1">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
@@ -1150,50 +1400,50 @@
         <v>5</v>
       </c>
       <c r="H19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>67057900414</v>
+        <v>67057900458</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C20" s="1">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="D20" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="F20" t="s">
         <v>5</v>
       </c>
       <c r="G20" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H20" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>67057900444</v>
+        <v>67057900414</v>
       </c>
       <c r="B21" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C21" s="1">
         <v>3.5</v>
       </c>
       <c r="D21" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="E21" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="F21" t="s">
         <v>5</v>
@@ -1202,18 +1452,18 @@
         <v>7</v>
       </c>
       <c r="H21" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>67057900443</v>
+        <v>67057900444</v>
       </c>
       <c r="B22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C22" s="1">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="D22" t="s">
         <v>58</v>
@@ -1228,24 +1478,24 @@
         <v>7</v>
       </c>
       <c r="H22" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>67057900482</v>
+        <v>67057900443</v>
       </c>
       <c r="B23" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C23" s="1">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="D23" t="s">
         <v>58</v>
       </c>
       <c r="E23" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F23" t="s">
         <v>5</v>
@@ -1254,15 +1504,15 @@
         <v>7</v>
       </c>
       <c r="H23" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>67057900461</v>
+        <v>67057900482</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C24" s="1">
         <v>3.5</v>
@@ -1271,7 +1521,7 @@
         <v>58</v>
       </c>
       <c r="E24" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F24" t="s">
         <v>5</v>
@@ -1280,7 +1530,7 @@
         <v>7</v>
       </c>
       <c r="H24" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
@@ -1288,25 +1538,753 @@
         <v>67057900461</v>
       </c>
       <c r="B25" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D25" t="s">
+        <v>58</v>
+      </c>
+      <c r="E25" t="s">
+        <v>67</v>
+      </c>
+      <c r="F25" t="s">
+        <v>5</v>
+      </c>
+      <c r="G25" t="s">
+        <v>7</v>
+      </c>
+      <c r="H25" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>67057900210</v>
+      </c>
+      <c r="B26" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C26" s="1">
+        <v>99</v>
+      </c>
+      <c r="D26" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" t="s">
+        <v>77</v>
+      </c>
+      <c r="F26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G26" t="s">
+        <v>5</v>
+      </c>
+      <c r="H26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>67057900140</v>
+      </c>
+      <c r="B27" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="1">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" t="s">
+        <v>80</v>
+      </c>
+      <c r="F27" t="s">
+        <v>5</v>
+      </c>
+      <c r="G27" t="s">
+        <v>7</v>
+      </c>
+      <c r="H27" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>67057900130</v>
+      </c>
+      <c r="B28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" s="1">
+        <v>9</v>
+      </c>
+      <c r="D28" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28" t="s">
+        <v>83</v>
+      </c>
+      <c r="F28" t="s">
+        <v>5</v>
+      </c>
+      <c r="G28" t="s">
+        <v>7</v>
+      </c>
+      <c r="H28" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>67057900301</v>
+      </c>
+      <c r="B29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" s="1">
+        <v>7</v>
+      </c>
+      <c r="D29" t="s">
+        <v>78</v>
+      </c>
+      <c r="E29" t="s">
+        <v>86</v>
+      </c>
+      <c r="F29" t="s">
+        <v>5</v>
+      </c>
+      <c r="G29" t="s">
+        <v>7</v>
+      </c>
+      <c r="H29" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>67057900495</v>
+      </c>
+      <c r="B30" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" s="1">
+        <v>6</v>
+      </c>
+      <c r="D30" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" t="s">
+        <v>89</v>
+      </c>
+      <c r="F30" t="s">
+        <v>5</v>
+      </c>
+      <c r="G30" t="s">
+        <v>7</v>
+      </c>
+      <c r="H30" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>67057900488</v>
+      </c>
+      <c r="B31" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="1">
+        <v>6</v>
+      </c>
+      <c r="D31" t="s">
+        <v>26</v>
+      </c>
+      <c r="E31" t="s">
+        <v>92</v>
+      </c>
+      <c r="F31" t="s">
+        <v>5</v>
+      </c>
+      <c r="G31" t="s">
+        <v>7</v>
+      </c>
+      <c r="H31" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>67057900472</v>
+      </c>
+      <c r="B32" t="s">
+        <v>94</v>
+      </c>
+      <c r="C32" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D32" t="s">
+        <v>26</v>
+      </c>
+      <c r="E32" t="s">
+        <v>95</v>
+      </c>
+      <c r="F32" t="s">
+        <v>5</v>
+      </c>
+      <c r="G32" t="s">
+        <v>7</v>
+      </c>
+      <c r="H32" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>67057900431</v>
+      </c>
+      <c r="B33" t="s">
+        <v>97</v>
+      </c>
+      <c r="C33" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D33" t="s">
+        <v>26</v>
+      </c>
+      <c r="E33" t="s">
+        <v>98</v>
+      </c>
+      <c r="F33" t="s">
+        <v>5</v>
+      </c>
+      <c r="G33" t="s">
+        <v>7</v>
+      </c>
+      <c r="H33" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>67057900463</v>
+      </c>
+      <c r="B34" t="s">
+        <v>100</v>
+      </c>
+      <c r="C34" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D34" t="s">
+        <v>26</v>
+      </c>
+      <c r="E34" t="s">
+        <v>101</v>
+      </c>
+      <c r="F34" t="s">
+        <v>5</v>
+      </c>
+      <c r="G34" t="s">
+        <v>7</v>
+      </c>
+      <c r="H34" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>67057900470</v>
+      </c>
+      <c r="B35" t="s">
+        <v>103</v>
+      </c>
+      <c r="C35" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D35" t="s">
+        <v>26</v>
+      </c>
+      <c r="E35" t="s">
+        <v>104</v>
+      </c>
+      <c r="F35" t="s">
+        <v>5</v>
+      </c>
+      <c r="G35" t="s">
+        <v>7</v>
+      </c>
+      <c r="H35" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>67057900427</v>
+      </c>
+      <c r="B36" t="s">
+        <v>106</v>
+      </c>
+      <c r="C36" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D36" t="s">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>107</v>
+      </c>
+      <c r="F36" t="s">
+        <v>5</v>
+      </c>
+      <c r="G36" t="s">
+        <v>7</v>
+      </c>
+      <c r="H36" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>67057900464</v>
+      </c>
+      <c r="B37" t="s">
+        <v>109</v>
+      </c>
+      <c r="C37" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D37" t="s">
+        <v>33</v>
+      </c>
+      <c r="E37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F37" t="s">
+        <v>5</v>
+      </c>
+      <c r="G37" t="s">
+        <v>7</v>
+      </c>
+      <c r="H37" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>67057900460</v>
+      </c>
+      <c r="B38" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D38" t="s">
+        <v>22</v>
+      </c>
+      <c r="E38" t="s">
+        <v>114</v>
+      </c>
+      <c r="F38" t="s">
+        <v>5</v>
+      </c>
+      <c r="G38" t="s">
+        <v>7</v>
+      </c>
+      <c r="H38" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>67057900417</v>
+      </c>
+      <c r="B39" t="s">
+        <v>116</v>
+      </c>
+      <c r="C39" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D39" t="s">
+        <v>22</v>
+      </c>
+      <c r="E39" t="s">
+        <v>117</v>
+      </c>
+      <c r="F39" t="s">
+        <v>5</v>
+      </c>
+      <c r="G39" t="s">
+        <v>7</v>
+      </c>
+      <c r="H39" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>67057900418</v>
+      </c>
+      <c r="B40" t="s">
+        <v>119</v>
+      </c>
+      <c r="C40" s="1">
+        <v>6</v>
+      </c>
+      <c r="D40" t="s">
+        <v>22</v>
+      </c>
+      <c r="E40" t="s">
+        <v>120</v>
+      </c>
+      <c r="F40" t="s">
+        <v>5</v>
+      </c>
+      <c r="G40" t="s">
+        <v>7</v>
+      </c>
+      <c r="H40" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>67057900445</v>
+      </c>
+      <c r="B41" t="s">
+        <v>124</v>
+      </c>
+      <c r="C41" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D41" t="s">
+        <v>58</v>
+      </c>
+      <c r="E41" t="s">
+        <v>122</v>
+      </c>
+      <c r="F41" t="s">
+        <v>5</v>
+      </c>
+      <c r="G41" t="s">
+        <v>7</v>
+      </c>
+      <c r="H41" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>67057900466</v>
+      </c>
+      <c r="B42" t="s">
+        <v>125</v>
+      </c>
+      <c r="C42" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D42" t="s">
+        <v>58</v>
+      </c>
+      <c r="E42" t="s">
+        <v>126</v>
+      </c>
+      <c r="F42" t="s">
+        <v>5</v>
+      </c>
+      <c r="G42" t="s">
+        <v>7</v>
+      </c>
+      <c r="H42" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>67057900462</v>
+      </c>
+      <c r="B43" t="s">
+        <v>128</v>
+      </c>
+      <c r="C43" s="1">
+        <v>6</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>129</v>
+      </c>
+      <c r="F43" t="s">
+        <v>5</v>
+      </c>
+      <c r="G43" t="s">
+        <v>7</v>
+      </c>
+      <c r="H43" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>67057900480</v>
+      </c>
+      <c r="B44" t="s">
+        <v>131</v>
+      </c>
+      <c r="C44" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="D44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E44" t="s">
+        <v>142</v>
+      </c>
+      <c r="F44" t="s">
+        <v>5</v>
+      </c>
+      <c r="G44" t="s">
+        <v>7</v>
+      </c>
+      <c r="H44" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>67057900481</v>
+      </c>
+      <c r="B45" t="s">
+        <v>133</v>
+      </c>
+      <c r="C45" s="1">
+        <v>10</v>
+      </c>
+      <c r="D45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45" t="s">
+        <v>142</v>
+      </c>
+      <c r="F45" t="s">
+        <v>5</v>
+      </c>
+      <c r="G45" t="s">
+        <v>7</v>
+      </c>
+      <c r="H45" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>67057900900</v>
+      </c>
+      <c r="B46" t="s">
+        <v>134</v>
+      </c>
+      <c r="C46" s="1">
+        <v>5</v>
+      </c>
+      <c r="D46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E46" t="s">
+        <v>141</v>
+      </c>
+      <c r="F46" t="s">
+        <v>5</v>
+      </c>
+      <c r="G46" t="s">
+        <v>5</v>
+      </c>
+      <c r="H46" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>67057900910</v>
+      </c>
+      <c r="B47" t="s">
+        <v>135</v>
+      </c>
+      <c r="C47" s="1">
+        <v>5</v>
+      </c>
+      <c r="D47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47" t="s">
+        <v>146</v>
+      </c>
+      <c r="F47" t="s">
+        <v>5</v>
+      </c>
+      <c r="G47" t="s">
+        <v>5</v>
+      </c>
+      <c r="H47" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>67057900407</v>
+      </c>
+      <c r="B48" t="s">
+        <v>145</v>
+      </c>
+      <c r="C48" s="1">
+        <v>5.99</v>
+      </c>
+      <c r="D48" t="s">
+        <v>22</v>
+      </c>
+      <c r="E48" t="s">
+        <v>147</v>
+      </c>
+      <c r="F48" t="s">
+        <v>5</v>
+      </c>
+      <c r="G48" t="s">
+        <v>7</v>
+      </c>
+      <c r="H48" t="s">
         <v>150</v>
       </c>
-      <c r="D25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E25" t="s">
-        <v>77</v>
-      </c>
-      <c r="F25" t="s">
-        <v>5</v>
-      </c>
-      <c r="G25" t="s">
-        <v>5</v>
-      </c>
-      <c r="H25" t="s">
-        <v>78</v>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>67057900225</v>
+      </c>
+      <c r="B49" t="s">
+        <v>143</v>
+      </c>
+      <c r="C49" s="1">
+        <v>5.99</v>
+      </c>
+      <c r="D49" t="s">
+        <v>12</v>
+      </c>
+      <c r="E49" t="s">
+        <v>158</v>
+      </c>
+      <c r="F49" t="s">
+        <v>5</v>
+      </c>
+      <c r="G49" t="s">
+        <v>7</v>
+      </c>
+      <c r="H49" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>67057900250</v>
+      </c>
+      <c r="B50" t="s">
+        <v>140</v>
+      </c>
+      <c r="C50" s="1">
+        <v>9.99</v>
+      </c>
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" t="s">
+        <v>161</v>
+      </c>
+      <c r="F50" t="s">
+        <v>5</v>
+      </c>
+      <c r="G50" t="s">
+        <v>7</v>
+      </c>
+      <c r="H50" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>67057900491</v>
+      </c>
+      <c r="B51" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" s="1">
+        <v>1.99</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>148</v>
+      </c>
+      <c r="F51" t="s">
+        <v>5</v>
+      </c>
+      <c r="G51" t="s">
+        <v>7</v>
+      </c>
+      <c r="H51" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>67057900497</v>
+      </c>
+      <c r="B52" t="s">
+        <v>136</v>
+      </c>
+      <c r="C52" s="1">
+        <v>2.4900000000000002</v>
+      </c>
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" t="s">
+        <v>160</v>
+      </c>
+      <c r="F52" t="s">
+        <v>5</v>
+      </c>
+      <c r="G52" t="s">
+        <v>7</v>
+      </c>
+      <c r="H52" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>67057900498</v>
+      </c>
+      <c r="B53" t="s">
+        <v>157</v>
+      </c>
+      <c r="C53" s="1">
+        <v>19.989999999999998</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>159</v>
+      </c>
+      <c r="F53" t="s">
+        <v>5</v>
+      </c>
+      <c r="G53" t="s">
+        <v>7</v>
+      </c>
+      <c r="H53" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>